<commit_message>
fix(data): restore https scheme on PPG careers URL
</commit_message>
<xml_diff>
--- a/data/input/master-input_companies.xlsx
+++ b/data/input/master-input_companies.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/alirizabagci/Documents/04_Projekte_Code/Python Projects/Upwork/singapore_ats_scraping/data/input/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FF5BDF42-A343-8C45-A4B5-279E676E14AF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9158D043-D927-614B-B3E8-440B4BDEDF01}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15760" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1952,7 +1952,7 @@
     <t xml:space="preserve">BP </t>
   </si>
   <si>
-    <t>careers.ppg.com/us/en/search-results?m=3&amp;location=Singapore%2C%20North%20East</t>
+    <t>https://careers.ppg.com/us/en/search-results?m=3&amp;location=Singapore%2C%20North%20East</t>
   </si>
 </sst>
 </file>
@@ -6225,7 +6225,7 @@
     <hyperlink ref="C211" r:id="rId10" xr:uid="{86951D57-E9F7-0748-B05B-BDA9DDD2F952}"/>
     <hyperlink ref="C218" r:id="rId11" xr:uid="{756CBA95-0C00-FC4F-BB97-C8F7DE6F7A86}"/>
     <hyperlink ref="C7" r:id="rId12" xr:uid="{881B0FEB-2F14-6840-A8C8-1C92F83887E2}"/>
-    <hyperlink ref="C55" r:id="rId13" display="https://careers.ppg.com/us/en/search-results?m=3&amp;location=Singapore%2C%20North%20East%2C%20Singapore" xr:uid="{948C709D-E26C-6B47-AF08-DB3D9D0B7ACF}"/>
+    <hyperlink ref="C55" r:id="rId13" xr:uid="{948C709D-E26C-6B47-AF08-DB3D9D0B7ACF}"/>
     <hyperlink ref="B79" r:id="rId14" xr:uid="{0102135B-8EA0-B04C-96D2-5C35A558E601}"/>
     <hyperlink ref="C79" r:id="rId15" xr:uid="{664F1B2F-018B-F840-AF0A-CA31BD6351AA}"/>
   </hyperlinks>

</xml_diff>